<commit_message>
Update timestamps and student assignments
Refresh generatedAt timestamps and update student data. annualEvents.json and students.json generatedAt fields updated. students.json contains many corrections to student block entries: subject/level swaps (HL/SL), teacher and room reassignments, additions/removals of blocks and extras (e.g., added TOK/TOK, moved Math/Global Politics/Biology/ESS entries), and other class name adjustments. The binary IB2 Class list 2025-2026.xlsx was also updated as a source for these changes.
</commit_message>
<xml_diff>
--- a/IB2 Class list 2025-2026.xlsx
+++ b/IB2 Class list 2025-2026.xlsx
@@ -2054,8 +2054,8 @@
         <v>4</v>
       </c>
       <c r="Z6" s="8">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.0)</f>
-        <v>16</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.0)</f>
+        <v>15</v>
       </c>
       <c r="AA6" s="8">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),3.0)</f>
@@ -2082,8 +2082,8 @@
         <v>11</v>
       </c>
       <c r="AG6" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
+        <v>9</v>
       </c>
       <c r="AH6" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.0)</f>
@@ -2126,8 +2126,8 @@
         <v>4</v>
       </c>
       <c r="AR6" s="2">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.0)</f>
-        <v>16</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.0)</f>
+        <v>15</v>
       </c>
       <c r="AS6" s="2">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11.0)</f>
@@ -2194,8 +2194,8 @@
         <v>8</v>
       </c>
       <c r="BI6" s="8">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),17.0)</f>
-        <v>17</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.0)</f>
+        <v>16</v>
       </c>
       <c r="BJ6" s="8">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.0)</f>
@@ -2210,8 +2210,8 @@
         <v>20</v>
       </c>
       <c r="BM6" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11.0)</f>
-        <v>11</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.0)</f>
+        <v>10</v>
       </c>
       <c r="BN6" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12.0)</f>
@@ -2313,8 +2313,8 @@
       </c>
       <c r="Y7" s="4"/>
       <c r="Z7" s="25">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),19.0)</f>
-        <v>19</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),18.0)</f>
+        <v>18</v>
       </c>
       <c r="AA7" s="4"/>
       <c r="AB7" s="7">
@@ -2335,8 +2335,8 @@
         <v>11</v>
       </c>
       <c r="AG7" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),8.0)</f>
-        <v>8</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),9.0)</f>
+        <v>9</v>
       </c>
       <c r="AH7" s="10">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),18.0)</f>
@@ -2367,8 +2367,8 @@
         <v>4</v>
       </c>
       <c r="AR7" s="2">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.0)</f>
-        <v>16</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),15.0)</f>
+        <v>15</v>
       </c>
       <c r="AS7" s="2">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11.0)</f>
@@ -2435,8 +2435,8 @@
         <v>8</v>
       </c>
       <c r="BI7" s="8">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),17.0)</f>
-        <v>17</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.0)</f>
+        <v>16</v>
       </c>
       <c r="BJ7" s="8">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),16.0)</f>
@@ -2451,8 +2451,8 @@
         <v>20</v>
       </c>
       <c r="BM7" s="9">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),11.0)</f>
-        <v>11</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),10.0)</f>
+        <v>10</v>
       </c>
       <c r="BN7" s="9">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),12.0)</f>
@@ -2715,7 +2715,10 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aarush Kumar")</f>
         <v>Aarush Kumar</v>
       </c>
-      <c r="BM8" s="39"/>
+      <c r="BM8" s="39" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aye Chan        Pyae Zone")</f>
+        <v>Aye Chan        Pyae Zone</v>
+      </c>
       <c r="BN8" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aarush Kumar")</f>
         <v>Aarush Kumar</v>
@@ -2827,10 +2830,7 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ximena Rosalyn	Ventura Diaz")</f>
         <v>Ximena Rosalyn	Ventura Diaz</v>
       </c>
-      <c r="Z9" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Cecilie Miklasz Carstensen")</f>
-        <v>Cecilie Miklasz Carstensen</v>
-      </c>
+      <c r="Z9" s="36"/>
       <c r="AA9" s="36" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Eain	Pyae")</f>
         <v>Eain	Pyae</v>
@@ -2974,7 +2974,10 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Cecilie Miklasz Carstensen")</f>
         <v>Cecilie Miklasz Carstensen</v>
       </c>
-      <c r="BM9" s="39"/>
+      <c r="BM9" s="39" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Berber        de Greef")</f>
+        <v>Berber        de Greef</v>
+      </c>
       <c r="BN9" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aunati        Kumar")</f>
         <v>Aunati        Kumar</v>
@@ -3213,8 +3216,8 @@
         <v>Chieh-Ni (Janice) Yang</v>
       </c>
       <c r="BM10" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aye Chan        Pyae Zone")</f>
-        <v>Aye Chan        Pyae Zone</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jules	Melgaard")</f>
+        <v>Jules	Melgaard</v>
       </c>
       <c r="BN10" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Azure        Adams")</f>
@@ -3451,8 +3454,8 @@
         <v>Aunati        Kumar</v>
       </c>
       <c r="BM11" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Berber        de Greef")</f>
-        <v>Berber        de Greef</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ronja	Grundig")</f>
+        <v>Ronja	Grundig</v>
       </c>
       <c r="BN11" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Danielle        Namuwonge")</f>
@@ -3684,10 +3687,13 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Kiran        Wilcke")</f>
         <v>Kiran        Wilcke</v>
       </c>
-      <c r="BL12" s="48"/>
+      <c r="BL12" s="48" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Berber        de Greef")</f>
+        <v>Berber        de Greef</v>
+      </c>
       <c r="BM12" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jules	Melgaard")</f>
-        <v>Jules	Melgaard</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isabel        Canas-Ferreira Daltrop")</f>
+        <v>Isabel        Canas-Ferreira Daltrop</v>
       </c>
       <c r="BN12" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Josie May	Thomas")</f>
@@ -3905,12 +3911,12 @@
       </c>
       <c r="BK13" s="48"/>
       <c r="BL13" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Berber        de Greef")</f>
-        <v>Berber        de Greef</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Federico        Corda")</f>
+        <v>Federico        Corda</v>
       </c>
       <c r="BM13" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Lucrezia Blanca	Morra")</f>
-        <v>Lucrezia Blanca	Morra</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ulrich	Mohrhdart Doger")</f>
+        <v>Ulrich	Mohrhdart Doger</v>
       </c>
       <c r="BN13" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Kelzang	Tobgyel")</f>
@@ -4125,10 +4131,13 @@
         <v>Pedro        Ortuño García</v>
       </c>
       <c r="BL14" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Federico        Corda")</f>
-        <v>Federico        Corda</v>
-      </c>
-      <c r="BM14" s="39"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Filip        Suchanski")</f>
+        <v>Filip        Suchanski</v>
+      </c>
+      <c r="BM14" s="39" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aoife Jassami Wade")</f>
+        <v>Aoife Jassami Wade</v>
+      </c>
       <c r="BN14" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Kris Xavier	Sealy")</f>
         <v>Kris Xavier	Sealy</v>
@@ -4336,12 +4345,12 @@
         <v>Lucrezia Blanca        Morra</v>
       </c>
       <c r="BL15" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Filip        Suchanski")</f>
-        <v>Filip        Suchanski</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Florenz Levian        Krauß")</f>
+        <v>Florenz Levian        Krauß</v>
       </c>
       <c r="BM15" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ronja	Grundig")</f>
-        <v>Ronja	Grundig</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Nguyen (Vivienne) Thao Phuong")</f>
+        <v>Nguyen (Vivienne) Thao Phuong</v>
       </c>
       <c r="BN15" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Oluwafamisoke Oluwadunbarin	Olatunbosun")</f>
@@ -4449,7 +4458,10 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pia  de Ville de Goyet")</f>
         <v>Pia  de Ville de Goyet</v>
       </c>
-      <c r="AG16" s="39"/>
+      <c r="AG16" s="39" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pia        de Ville de Goyet")</f>
+        <v>Pia        de Ville de Goyet</v>
+      </c>
       <c r="AH16" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Klaudia	Wyrębkowska")</f>
         <v>Klaudia	Wyrębkowska</v>
@@ -4535,12 +4547,12 @@
         <v>Pia  de Ville de Goyet</v>
       </c>
       <c r="BL16" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Florenz Levian        Krauß")</f>
-        <v>Florenz Levian        Krauß</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jade Yixuan        Wang")</f>
+        <v>Jade Yixuan        Wang</v>
       </c>
       <c r="BM16" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isabel        Canas-Ferreira Daltrop")</f>
-        <v>Isabel        Canas-Ferreira Daltrop</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pamela	Solís Arias")</f>
+        <v>Pamela	Solís Arias</v>
       </c>
       <c r="BN16" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Tenzin	Jigme")</f>
@@ -4713,8 +4725,8 @@
       </c>
       <c r="BH17" s="78"/>
       <c r="BI17" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Maitreyi Manoj        Nair")</f>
-        <v>Maitreyi Manoj        Nair</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Nguyen Thao        Phuong")</f>
+        <v>Nguyen Thao        Phuong</v>
       </c>
       <c r="BJ17" s="36" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pamela        Solís Arias")</f>
@@ -4725,12 +4737,12 @@
         <v>Min Fu (Mark)        Huang</v>
       </c>
       <c r="BL17" s="52" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jade Yixuan        Wang")</f>
-        <v>Jade Yixuan        Wang</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Josie May        Thomas")</f>
+        <v>Josie May        Thomas</v>
       </c>
       <c r="BM17" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ulrich	Mohrhdart Doger")</f>
-        <v>Ulrich	Mohrhdart Doger</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Yao Wei	Zheng He")</f>
+        <v>Yao Wei	Zheng He</v>
       </c>
       <c r="BN17" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aryaka        Bist")</f>
@@ -4885,8 +4897,8 @@
       <c r="BG18" s="82"/>
       <c r="BH18" s="48"/>
       <c r="BI18" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Nguyen Thao        Phuong")</f>
-        <v>Nguyen Thao        Phuong</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Olivia        Moe-Jordan")</f>
+        <v>Olivia        Moe-Jordan</v>
       </c>
       <c r="BJ18" s="36" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Rosmeily de Jesús        Reyes")</f>
@@ -4897,8 +4909,8 @@
         <v>Naya        Niedermayr</v>
       </c>
       <c r="BL18" s="66" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Josie May        Thomas")</f>
-        <v>Josie May        Thomas</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jules        Melgaard")</f>
+        <v>Jules        Melgaard</v>
       </c>
       <c r="BM18" s="39"/>
       <c r="BN18" s="38" t="str">
@@ -5051,8 +5063,8 @@
       <c r="BG19" s="82"/>
       <c r="BH19" s="48"/>
       <c r="BI19" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Olivia        Moe-Jordan")</f>
-        <v>Olivia        Moe-Jordan</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sofia        Tomasikova")</f>
+        <v>Sofia        Tomasikova</v>
       </c>
       <c r="BJ19" s="36" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ximena Rosalyn        Ventura Diaz")</f>
@@ -5060,13 +5072,10 @@
       </c>
       <c r="BK19" s="82"/>
       <c r="BL19" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jules        Melgaard")</f>
-        <v>Jules        Melgaard</v>
-      </c>
-      <c r="BM19" s="79" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Aoife Jassami Wade")</f>
-        <v>Aoife Jassami Wade</v>
-      </c>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Kris Xavier        Sealy")</f>
+        <v>Kris Xavier        Sealy</v>
+      </c>
+      <c r="BM19" s="79"/>
       <c r="BN19" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ventsislav	Dinkov")</f>
         <v>Ventsislav	Dinkov</v>
@@ -5205,19 +5214,19 @@
       <c r="BG20" s="89"/>
       <c r="BH20" s="48"/>
       <c r="BI20" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sofia        Tomasikova")</f>
-        <v>Sofia        Tomasikova</v>
-      </c>
-      <c r="BJ20" s="48"/>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Tilda        Gaspar")</f>
+        <v>Tilda        Gaspar</v>
+      </c>
+      <c r="BJ20" s="48" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Kristhel Gabriela        Ayapán Balcárcel")</f>
+        <v>Kristhel Gabriela        Ayapán Balcárcel</v>
+      </c>
       <c r="BK20" s="90"/>
       <c r="BL20" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Kris Xavier        Sealy")</f>
-        <v>Kris Xavier        Sealy</v>
-      </c>
-      <c r="BM20" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Nguyen (Vivienne) Thao Phuong")</f>
-        <v>Nguyen (Vivienne) Thao Phuong</v>
-      </c>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Laora        Servant")</f>
+        <v>Laora        Servant</v>
+      </c>
+      <c r="BM20" s="38"/>
       <c r="BN20" s="57"/>
       <c r="BO20" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Hedda        Olson")</f>
@@ -5312,8 +5321,8 @@
       <c r="AP21" s="39"/>
       <c r="AQ21" s="39"/>
       <c r="AR21" s="31" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pia        de Ville de Goyet")</f>
-        <v>Pia        de Ville de Goyet</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Tahmina        Tamim")</f>
+        <v>Tahmina        Tamim</v>
       </c>
       <c r="AS21" s="30"/>
       <c r="AT21" s="30"/>
@@ -5344,22 +5353,19 @@
       <c r="BG21" s="50"/>
       <c r="BH21" s="48"/>
       <c r="BI21" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Tilda        Gaspar")</f>
-        <v>Tilda        Gaspar</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Xiaoshi (Stone)        ZHAO")</f>
+        <v>Xiaoshi (Stone)        ZHAO</v>
       </c>
       <c r="BJ21" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Kristhel Gabriela        Ayapán Balcárcel")</f>
-        <v>Kristhel Gabriela        Ayapán Balcárcel</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Emely Johanya        López Torres")</f>
+        <v>Emely Johanya        López Torres</v>
       </c>
       <c r="BK21" s="82"/>
       <c r="BL21" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Laora        Servant")</f>
-        <v>Laora        Servant</v>
-      </c>
-      <c r="BM21" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Pamela	Solís Arias")</f>
-        <v>Pamela	Solís Arias</v>
-      </c>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sophia        Gehann")</f>
+        <v>Sophia        Gehann</v>
+      </c>
+      <c r="BM21" s="38"/>
       <c r="BN21" s="39"/>
       <c r="BO21" s="38" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Tara        van Wijk")</f>
@@ -5447,10 +5453,7 @@
       <c r="AO22" s="39"/>
       <c r="AP22" s="39"/>
       <c r="AQ22" s="39"/>
-      <c r="AR22" s="31" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Tahmina        Tamim")</f>
-        <v>Tahmina        Tamim</v>
-      </c>
+      <c r="AR22" s="31"/>
       <c r="AS22" s="30"/>
       <c r="AT22" s="30"/>
       <c r="AU22" s="31" t="str">
@@ -5480,22 +5483,19 @@
       <c r="BG22" s="48"/>
       <c r="BH22" s="48"/>
       <c r="BI22" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Xiaoshi (Stone)        ZHAO")</f>
-        <v>Xiaoshi (Stone)        ZHAO</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Yao Wei        Zheng He")</f>
+        <v>Yao Wei        Zheng He</v>
       </c>
       <c r="BJ22" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Emely Johanya        López Torres")</f>
-        <v>Emely Johanya        López Torres</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ulrich        Mohrhdart Doger")</f>
+        <v>Ulrich        Mohrhdart Doger</v>
       </c>
       <c r="BK22" s="50"/>
       <c r="BL22" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Sophia        Gehann")</f>
-        <v>Sophia        Gehann</v>
-      </c>
-      <c r="BM22" s="38" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Yao Wei	Zheng He")</f>
-        <v>Yao Wei	Zheng He</v>
-      </c>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isabela        Aurélio de Vargas")</f>
+        <v>Isabela        Aurélio de Vargas</v>
+      </c>
+      <c r="BM22" s="38"/>
       <c r="BN22" s="39"/>
       <c r="BO22" s="61" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Zoé Sara	Amat")</f>
@@ -5574,7 +5574,10 @@
       <c r="AO23" s="55"/>
       <c r="AP23" s="39"/>
       <c r="AQ23" s="39"/>
-      <c r="AR23" s="30"/>
+      <c r="AR23" s="30" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Zoé Sara        Amat")</f>
+        <v>Zoé Sara        Amat</v>
+      </c>
       <c r="AS23" s="30"/>
       <c r="AT23" s="30"/>
       <c r="AU23" s="31" t="str">
@@ -5604,17 +5607,17 @@
       <c r="BG23" s="48"/>
       <c r="BH23" s="48"/>
       <c r="BI23" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Yao Wei        Zheng He")</f>
-        <v>Yao Wei        Zheng He</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Alejandro Daniel Portillo Cabral")</f>
+        <v>Alejandro Daniel Portillo Cabral</v>
       </c>
       <c r="BJ23" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Ulrich        Mohrhdart Doger")</f>
-        <v>Ulrich        Mohrhdart Doger</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jorge Alexander        Rivero Añez")</f>
+        <v>Jorge Alexander        Rivero Añez</v>
       </c>
       <c r="BK23" s="48"/>
       <c r="BL23" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Isabela        Aurélio de Vargas")</f>
-        <v>Isabela        Aurélio de Vargas</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Tahmina        Tamim")</f>
+        <v>Tahmina        Tamim</v>
       </c>
       <c r="BM23" s="57"/>
       <c r="BN23" s="39"/>
@@ -5690,8 +5693,8 @@
       <c r="AP24" s="39"/>
       <c r="AQ24" s="39"/>
       <c r="AR24" s="31" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Zoé Sara        Amat")</f>
-        <v>Zoé Sara        Amat</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Alina Araya Hernández")</f>
+        <v>Alina Araya Hernández</v>
       </c>
       <c r="AS24" s="30"/>
       <c r="AT24" s="30"/>
@@ -5718,18 +5721,12 @@
       <c r="BF24" s="48"/>
       <c r="BG24" s="48"/>
       <c r="BH24" s="48"/>
-      <c r="BI24" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Alejandro Daniel Portillo Cabral")</f>
-        <v>Alejandro Daniel Portillo Cabral</v>
-      </c>
-      <c r="BJ24" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Jorge Alexander        Rivero Añez")</f>
-        <v>Jorge Alexander        Rivero Añez</v>
-      </c>
+      <c r="BI24" s="36"/>
+      <c r="BJ24" s="36"/>
       <c r="BK24" s="48"/>
       <c r="BL24" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Tahmina        Tamim")</f>
-        <v>Tahmina        Tamim</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Elba        de la Oliva")</f>
+        <v>Elba        de la Oliva</v>
       </c>
       <c r="BM24" s="39"/>
       <c r="BN24" s="39"/>
@@ -5793,8 +5790,8 @@
       <c r="AP25" s="39"/>
       <c r="AQ25" s="39"/>
       <c r="AR25" s="31" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Alina Araya Hernández")</f>
-        <v>Alina Araya Hernández</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Eddie Xi")</f>
+        <v>Eddie Xi</v>
       </c>
       <c r="AS25" s="30"/>
       <c r="AT25" s="30"/>
@@ -5822,8 +5819,8 @@
       <c r="BJ25" s="48"/>
       <c r="BK25" s="50"/>
       <c r="BL25" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Elba        de la Oliva")</f>
-        <v>Elba        de la Oliva</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Hsuan-Hao	Chang")</f>
+        <v>Hsuan-Hao	Chang</v>
       </c>
       <c r="BM25" s="39"/>
       <c r="BN25" s="39"/>
@@ -5889,10 +5886,7 @@
       <c r="AO26" s="39"/>
       <c r="AP26" s="39"/>
       <c r="AQ26" s="39"/>
-      <c r="AR26" s="51" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Eddie Xi")</f>
-        <v>Eddie Xi</v>
-      </c>
+      <c r="AR26" s="51"/>
       <c r="AS26" s="30"/>
       <c r="AT26" s="30"/>
       <c r="AU26" s="38" t="str">
@@ -5918,7 +5912,10 @@
       <c r="BI26" s="49"/>
       <c r="BJ26" s="48"/>
       <c r="BK26" s="48"/>
-      <c r="BL26" s="48"/>
+      <c r="BL26" s="48" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Arianna        Candeloro")</f>
+        <v>Arianna        Candeloro</v>
+      </c>
       <c r="BM26" s="39"/>
       <c r="BN26" s="39"/>
       <c r="BO26" s="39"/>
@@ -6007,8 +6004,8 @@
       <c r="BJ27" s="48"/>
       <c r="BK27" s="48"/>
       <c r="BL27" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Hsuan-Hao	Chang")</f>
-        <v>Hsuan-Hao	Chang</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Maxime        De Corioli")</f>
+        <v>Maxime        De Corioli</v>
       </c>
       <c r="BM27" s="39"/>
       <c r="BN27" s="39"/>
@@ -6091,10 +6088,7 @@
       <c r="BI28" s="48"/>
       <c r="BJ28" s="48"/>
       <c r="BK28" s="48"/>
-      <c r="BL28" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Arianna        Candeloro")</f>
-        <v>Arianna        Candeloro</v>
-      </c>
+      <c r="BL28" s="36"/>
       <c r="BM28" s="39"/>
       <c r="BN28" s="39"/>
       <c r="BO28" s="39"/>
@@ -6173,10 +6167,7 @@
       <c r="BI29" s="48"/>
       <c r="BJ29" s="48"/>
       <c r="BK29" s="48"/>
-      <c r="BL29" s="36" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Maxime        De Corioli")</f>
-        <v>Maxime        De Corioli</v>
-      </c>
+      <c r="BL29" s="36"/>
       <c r="BM29" s="39"/>
       <c r="BN29" s="39"/>
       <c r="BO29" s="39"/>

</xml_diff>